<commit_message>
Mismatch V1/V2 table: add combined-worst data + highlight worst deviation per column
</commit_message>
<xml_diff>
--- a/docs/mismatch_table_v1_v2.xlsx
+++ b/docs/mismatch_table_v1_v2.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,11 +43,15 @@
       <b val="1"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="008A1C1C"/>
+    </font>
+    <font>
       <i val="1"/>
       <color rgb="00666666"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -79,6 +83,11 @@
         <fgColor rgb="00D6E6F7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD24D"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -106,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -129,6 +138,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -141,7 +153,8 @@
     <xf numFmtId="164" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,10 +520,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
@@ -684,22 +697,22 @@
       <c r="C7" s="10" t="n">
         <v>1.2747</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="10" t="n">
         <v>0.1509</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="10" t="n">
         <v>0.3461</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="11" t="n">
         <v>0.3404</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="11" t="n">
         <v>0.3582</v>
       </c>
-      <c r="H7" s="11" t="n">
+      <c r="H7" s="12" t="n">
         <v>0.0546</v>
       </c>
-      <c r="I7" s="11" t="n">
+      <c r="I7" s="12" t="n">
         <v>0.1125</v>
       </c>
       <c r="J7" s="10" t="n">
@@ -708,10 +721,10 @@
       <c r="K7" s="10" t="n">
         <v>1.5571</v>
       </c>
-      <c r="L7" s="11" t="n">
+      <c r="L7" s="10" t="n">
         <v>0.1239</v>
       </c>
-      <c r="M7" s="11" t="n">
+      <c r="M7" s="10" t="n">
         <v>0.3835</v>
       </c>
     </row>
@@ -721,40 +734,40 @@
           <t>-10%</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="11" t="n">
         <v>0.5137</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="11" t="n">
         <v>0.5735</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="12" t="n">
         <v>0.0892</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="12" t="n">
         <v>0.1758</v>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="11" t="n">
         <v>0.1946</v>
       </c>
-      <c r="G8" s="10" t="n">
+      <c r="G8" s="11" t="n">
         <v>0.2095</v>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="H8" s="12" t="n">
         <v>0.0462</v>
       </c>
-      <c r="I8" s="11" t="n">
+      <c r="I8" s="12" t="n">
         <v>0.0823</v>
       </c>
-      <c r="J8" s="10" t="n">
+      <c r="J8" s="11" t="n">
         <v>0.408</v>
       </c>
-      <c r="K8" s="10" t="n">
+      <c r="K8" s="11" t="n">
         <v>0.4454</v>
       </c>
-      <c r="L8" s="11" t="n">
+      <c r="L8" s="12" t="n">
         <v>0.065</v>
       </c>
-      <c r="M8" s="11" t="n">
+      <c r="M8" s="12" t="n">
         <v>0.1598</v>
       </c>
     </row>
@@ -764,40 +777,40 @@
           <t>0%</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="13" t="n">
         <v>0.0286</v>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="13" t="n">
         <v>0.0306</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="14" t="n">
         <v>0.0436</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="14" t="n">
         <v>0.0552</v>
       </c>
-      <c r="F9" s="12" t="n">
+      <c r="F9" s="13" t="n">
         <v>0.0286</v>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="G9" s="13" t="n">
         <v>0.0306</v>
       </c>
-      <c r="H9" s="13" t="n">
+      <c r="H9" s="14" t="n">
         <v>0.0436</v>
       </c>
-      <c r="I9" s="13" t="n">
+      <c r="I9" s="14" t="n">
         <v>0.0552</v>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="13" t="n">
         <v>0.0286</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="K9" s="13" t="n">
         <v>0.0306</v>
       </c>
-      <c r="L9" s="13" t="n">
+      <c r="L9" s="14" t="n">
         <v>0.0436</v>
       </c>
-      <c r="M9" s="13" t="n">
+      <c r="M9" s="14" t="n">
         <v>0.0552</v>
       </c>
     </row>
@@ -807,40 +820,40 @@
           <t>+10%</t>
         </is>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="11" t="n">
         <v>0.4486</v>
       </c>
-      <c r="C10" s="10" t="n">
+      <c r="C10" s="11" t="n">
         <v>0.4416</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="12" t="n">
         <v>0.0679</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="12" t="n">
         <v>0.08400000000000001</v>
       </c>
-      <c r="F10" s="10" t="n">
+      <c r="F10" s="11" t="n">
         <v>0.3334</v>
       </c>
-      <c r="G10" s="10" t="n">
+      <c r="G10" s="11" t="n">
         <v>0.3692</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H10" s="12" t="n">
         <v>0.0615</v>
       </c>
-      <c r="I10" s="11" t="n">
+      <c r="I10" s="12" t="n">
         <v>0.1424</v>
       </c>
-      <c r="J10" s="10" t="n">
+      <c r="J10" s="11" t="n">
         <v>0.1796</v>
       </c>
-      <c r="K10" s="10" t="n">
+      <c r="K10" s="11" t="n">
         <v>0.1936</v>
       </c>
-      <c r="L10" s="11" t="n">
+      <c r="L10" s="12" t="n">
         <v>0.0454</v>
       </c>
-      <c r="M10" s="11" t="n">
+      <c r="M10" s="12" t="n">
         <v>0.07829999999999999</v>
       </c>
     </row>
@@ -850,16 +863,16 @@
           <t>+20%</t>
         </is>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="11" t="n">
         <v>0.8493000000000001</v>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="11" t="n">
         <v>0.7783</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="12" t="n">
         <v>0.1068</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="12" t="n">
         <v>0.1119</v>
       </c>
       <c r="F11" s="10" t="n">
@@ -868,29 +881,75 @@
       <c r="G11" s="10" t="n">
         <v>1.3349</v>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="H11" s="10" t="n">
         <v>0.1005</v>
       </c>
-      <c r="I11" s="11" t="n">
+      <c r="I11" s="10" t="n">
         <v>0.3069</v>
       </c>
-      <c r="J11" s="10" t="n">
+      <c r="J11" s="11" t="n">
         <v>0.2952</v>
       </c>
-      <c r="K11" s="10" t="n">
+      <c r="K11" s="11" t="n">
         <v>0.3132</v>
       </c>
-      <c r="L11" s="11" t="n">
+      <c r="L11" s="12" t="n">
         <v>0.0519</v>
       </c>
-      <c r="M11" s="11" t="n">
+      <c r="M11" s="12" t="n">
         <v>0.1034</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>Read-down each column: V1 (old) error grows steeply with deviation; V2 stays low = far more robust. 0% = nominal (no mismatch).</t>
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>COMBINED WORST</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>V1 meas</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>V1 hid</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>V2 meas</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>V2 hid</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>(m -20%, I +20%, l -20%)</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>3.0034</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>3.2302</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>0.3384</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>0.6963</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Amber = worst deviation in that column. Combined-worst combines each parameter's individually-worst direction. 0% = nominal.</t>
         </is>
       </c>
     </row>

</xml_diff>